<commit_message>
proposed changes to 2026/7
</commit_message>
<xml_diff>
--- a/AssessmentSchedule_2526_v2.xlsx
+++ b/AssessmentSchedule_2526_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cf-my.sharepoint.com/personal/northce_cardiff_ac_uk/Documents/Documents/Cardiff/DUGS/Assessments/Schedule Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1716" documentId="8_{10702854-9EE2-4D67-90CE-85FDD07A66EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49EEAAE0-471A-47C0-9AB3-B72E4BBA97EE}"/>
+  <xr:revisionPtr revIDLastSave="1719" documentId="8_{10702854-9EE2-4D67-90CE-85FDD07A66EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CBAF7FB-AB00-58E1-9A40-3A14ACFFFC85}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
+    <workbookView xWindow="5080" yWindow="5080" windowWidth="28800" windowHeight="15290" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Assessments" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId5"/>
+    <pivotCache cacheId="1" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -9045,7 +9045,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F344565-A902-475D-ACD8-7DA2FB255CBD}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F344565-A902-475D-ACD8-7DA2FB255CBD}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:B70" firstHeaderRow="1" firstDataRow="1" firstDataCol="2"/>
   <pivotFields count="34">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -9962,21 +9962,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66039B40-29AD-4D93-B125-EAF72A7B3996}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AL178"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.81640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.81640625" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" style="10" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="10" style="10" customWidth="1"/>
-    <col min="6" max="6" width="21.7109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="21.7109375" style="10" customWidth="1"/>
-    <col min="9" max="9" width="10.7109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="10.7109375" style="10" customWidth="1"/>
-    <col min="12" max="23" width="9.140625" style="14" customWidth="1"/>
-    <col min="24" max="36" width="9.140625" style="16"/>
+    <col min="6" max="6" width="21.7265625" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="21.7265625" style="10" customWidth="1"/>
+    <col min="9" max="9" width="10.7265625" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.7265625" style="10" customWidth="1"/>
+    <col min="12" max="23" width="9.1796875" style="14" customWidth="1"/>
+    <col min="24" max="36" width="9.1796875" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" s="44" customFormat="1" ht="30">
+    <row r="1" spans="1:38" s="44" customFormat="1" ht="29">
       <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
@@ -17061,7 +17061,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="92" spans="1:38" ht="28.5">
+    <row r="92" spans="1:38">
       <c r="A92" s="8" t="s">
         <v>21</v>
       </c>
@@ -17132,7 +17132,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="93" spans="1:38" ht="28.5">
+    <row r="93" spans="1:38">
       <c r="A93" s="8" t="s">
         <v>21</v>
       </c>
@@ -23648,16 +23648,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0482654D-1732-43E5-85EC-021407B07CE5}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AE141"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.81640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.81640625" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" style="10" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="10" style="10" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" style="10" customWidth="1"/>
-    <col min="7" max="15" width="16.28515625" style="14" bestFit="1" customWidth="1"/>
-    <col min="16" max="18" width="17.28515625" style="14" bestFit="1" customWidth="1"/>
-    <col min="19" max="30" width="8.7109375" style="16"/>
+    <col min="6" max="6" width="10.7265625" style="10" customWidth="1"/>
+    <col min="7" max="15" width="16.26953125" style="14" bestFit="1" customWidth="1"/>
+    <col min="16" max="18" width="17.26953125" style="14" bestFit="1" customWidth="1"/>
+    <col min="19" max="30" width="8.7265625" style="16"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31">
@@ -26979,7 +26979,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="1:31" ht="28.5">
+    <row r="36" spans="1:31">
       <c r="A36" s="8" t="s">
         <v>21</v>
       </c>
@@ -29803,14 +29803,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D548CE7-BEAC-43FA-847F-FDE82E3A5926}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:W129"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.81640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.81640625" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.85546875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.81640625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="10.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.26953125" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9" style="5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" style="5" customWidth="1"/>
   </cols>
@@ -31624,7 +31624,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:23" ht="28.5">
+    <row r="36" spans="1:23">
       <c r="A36" s="8" t="s">
         <v>21</v>
       </c>
@@ -35235,11 +35235,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF4F541C-C22C-46EF-BD21-4F8C93ABA5A9}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A3:F70"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="19.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="19.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:6">

</xml_diff>

<commit_message>
added PGT programmes, tweaks to schedules
</commit_message>
<xml_diff>
--- a/AssessmentSchedule_2526_v2.xlsx
+++ b/AssessmentSchedule_2526_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cf-my.sharepoint.com/personal/northce_cardiff_ac_uk/Documents/Documents/Cardiff/DUGS/Assessments/Schedule Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1719" documentId="8_{10702854-9EE2-4D67-90CE-85FDD07A66EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CBAF7FB-AB00-58E1-9A40-3A14ACFFFC85}"/>
+  <xr:revisionPtr revIDLastSave="1720" documentId="8_{10702854-9EE2-4D67-90CE-85FDD07A66EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12F72576-1D78-46D3-A873-4CF2A6818966}"/>
   <bookViews>
-    <workbookView xWindow="5080" yWindow="5080" windowWidth="28800" windowHeight="15290" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" activeTab="2" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Assessments" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId5"/>
+    <pivotCache cacheId="3" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -9045,7 +9045,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F344565-A902-475D-ACD8-7DA2FB255CBD}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F344565-A902-475D-ACD8-7DA2FB255CBD}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:B70" firstHeaderRow="1" firstDataRow="1" firstDataCol="2"/>
   <pivotFields count="34">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">

</xml_diff>